<commit_message>
Thermo-data for Cu111 corrected the vibrational frequency data for CHOHX
</commit_message>
<xml_diff>
--- a/Data/Cu111/vibrational_freq_zpe_Cu111.xlsx
+++ b/Data/Cu111/vibrational_freq_zpe_Cu111.xlsx
@@ -890,7 +890,9 @@
       <c r="M10" t="n">
         <v>102.601484</v>
       </c>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>57.682963</v>
+      </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
@@ -2053,30 +2055,32 @@
         <v>167.247947</v>
       </c>
       <c r="F32" t="n">
+        <v>145.810682</v>
+      </c>
+      <c r="G32" t="n">
         <v>129.130361</v>
       </c>
-      <c r="G32" t="n">
+      <c r="H32" t="n">
         <v>86.016997</v>
       </c>
-      <c r="H32" t="n">
+      <c r="I32" t="n">
         <v>52.982502</v>
       </c>
-      <c r="I32" t="n">
+      <c r="J32" t="n">
         <v>39.11396</v>
       </c>
-      <c r="J32" t="n">
+      <c r="K32" t="n">
         <v>28.726424</v>
       </c>
-      <c r="K32" t="n">
+      <c r="L32" t="n">
         <v>25.246032</v>
       </c>
-      <c r="L32" t="n">
+      <c r="M32" t="n">
         <v>12.720957</v>
       </c>
-      <c r="M32" t="n">
+      <c r="N32" t="n">
         <v>7.151773</v>
       </c>
-      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>

</xml_diff>